<commit_message>
Add whole blood as a sample type, and allow fractional ages
Whole blood is added to the template dropdown and, in the designer, to the
types it recognises, the types autofill places, the volume rules, and the
places that list the types to the user. A type the designer does not know is
flagged as unknown, never auto-filled and skipped by the volume check, so the
dropdown entry alone would not have worked.

Its volume rule is copied from serum and the note in the dialog says so — the
floor for whole blood has not been specified here.

subject_age_yrs now accepts decimals, for infants and for ages recorded to
part of a year.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBH1P2zpiSLx4BR7WKjhzK
</commit_message>
<xml_diff>
--- a/PhIPSeq_Manifest_Template_v5.xlsx
+++ b/PhIPSeq_Manifest_Template_v5.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Subject age in years at collection. Whole number, 0-120.</t>
+          <t>Subject age in years at collection, 0-120. Decimals allowed, for infants and for ages recorded to part of a year.</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>serum, plasma, CSF, mAb, control or assay control. serum/plasma/CSF are placed by autofill; the rest are placed by hand in the control area.</t>
+          <t>serum, plasma, whole blood, CSF, mAb, control or assay control. serum, plasma, whole blood and CSF are placed by autofill; the rest are placed by hand in the control area.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -3430,15 +3430,15 @@
     <dataValidation sqref="C3:C102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="subject_id" error="subject_id is required: tiu_id is built from sample_id and subject_id, and the designer uses it to keep one subject's samples on one plate." type="custom">
       <formula1>=LEN(TRIM($C3))&gt;0</formula1>
     </dataValidation>
-    <dataValidation sqref="D3:D102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="subject_age_yrs" error="Age must be a whole number of years between 0 and 120." type="whole" operator="between">
+    <dataValidation sqref="D3:D102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="subject_age_yrs" error="Age in years, between 0 and 120. Decimals are allowed — use them for infants and for ages recorded to part of a year (e.g. 0.5)." type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>120</formula2>
     </dataValidation>
     <dataValidation sqref="E3:E102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="subject_sex" error="Choose M, F or Unknown." type="list">
       <formula1>"M,F,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="sample_type" error="sample_type is required. serum, plasma and CSF are placed by autofill; mAb, control and assay control are placed by hand in the control area." type="list">
-      <formula1>"serum,plasma,CSF,mAb,control,assay control"</formula1>
+    <dataValidation sqref="G3:G102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="sample_type" error="sample_type is required. serum, plasma, whole blood and CSF are placed by autofill; mAb, control and assay control are placed by hand in the control area." type="list">
+      <formula1>"serum,plasma,whole blood,CSF,mAb,control,assay control"</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H102" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="volume_mL" error="Volume must be a positive number of millilitres (e.g. 0.5)." type="decimal" operator="greaterThan">
       <formula1>0</formula1>

</xml_diff>